<commit_message>
Update schedule details and speaker information for Endogineco 2026
- Corrected speaker names and affiliations in the schedule, including updates for Beethoven Landin and Kathiane Lustosa.
- Adjusted session timings and descriptions for clarity and consistency across HTML, CSV, and PDF formats.
- Enhanced the overall presentation of the schedule to ensure accurate information for attendees.
</commit_message>
<xml_diff>
--- a/endogineco2026/schedule/programacao-preliminar-2026.xlsx
+++ b/endogineco2026/schedule/programacao-preliminar-2026.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Programação CONGRESSO " sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Programação CONGRESSO '!$A$1:$C$127</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Programação CONGRESSO '!$A$1:$C$126</definedName>
   </definedNames>
   <calcPr/>
   <extLst>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="249">
   <si>
     <t xml:space="preserve"> CONGRESSO ENDOGINECO </t>
   </si>
@@ -272,7 +272,7 @@
         <color theme="3"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">Beethoven Landin - SP  </t>
+      <t xml:space="preserve">Beethoven Landin - CE  </t>
     </r>
     <r>
       <rPr>
@@ -504,7 +504,7 @@
 Kathiane Lustosa - CE, (ginecologista)
 Mayara Macedo -PE, (fisioterapeuta pelvica)
 Macira Sotero- PE, (psicóloga)
-Beethoven (coloproctologista)</t>
+Beethoven Landim - CE (coloproctologista)</t>
   </si>
   <si>
     <t>ENCERRAMENTO</t>
@@ -789,7 +789,7 @@
         <color theme="3"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">Bethoven Landin - SP</t>
+      <t xml:space="preserve">Bethoven Landin - CE</t>
     </r>
     <r>
       <rPr>
@@ -883,7 +883,7 @@
   <si>
     <t xml:space="preserve">MESA 1 - Infertilidade e Endometriose 
 Presidente: Agostinho Machado - PE 
-Debatedores: Hélio Costa - PE, Catarina Monteiro - PE , Eveline Catão - PE </t>
+Debatedores: Catarina Monteiro - PE , Eveline Catão - PE </t>
   </si>
   <si>
     <t xml:space="preserve">O que fazer primeiro na paciente com endometriose : FiV  antes e depois operar ou operar e depois a FIV ?</t>
@@ -1013,7 +1013,7 @@
 (20 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">SIMPÓSIO </t>
+    <t xml:space="preserve">INTERVALO LIVRE </t>
   </si>
   <si>
     <t xml:space="preserve">12:55 - 13:35
@@ -1084,7 +1084,7 @@
   <si>
     <t xml:space="preserve">MESA 2 - Coloproctologia no painel         
 Presidente : Marcos Saturnino - PE
-Debatedores: Beethoven Landin - PE, </t>
+Debatedores: Beethoven Landin - CE, Pedro Gonzaga - PE</t>
   </si>
   <si>
     <t xml:space="preserve">13:35 - 14:05            (30 min)
@@ -1156,7 +1156,7 @@
   </si>
   <si>
     <t xml:space="preserve">CIRURGIAS AO VIVO                                                                                                                                                                                        Coordenador : Jardel Soares - PE
-Debatedores : Sidraiton Melo - PE, Andreisa Bilhar - CE, Yole Minervino - PB</t>
+Debatedores : Sidraiton Melo - PE, Andreisa Bilhar - CE</t>
   </si>
   <si>
     <r>
@@ -1408,14 +1408,8 @@
 (10 min) </t>
   </si>
   <si>
-    <t xml:space="preserve">SIMPÓSIO (SALA A) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">12:55 - 13:40
-(45 min) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">INTERVALO LIVRE </t>
+    <t xml:space="preserve">12:35 - 13:40
+(01 hora e 05 min) </t>
   </si>
   <si>
     <t xml:space="preserve">13:40 - 14:20
@@ -1476,7 +1470,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11.000000"/>
       <color indexed="64"/>
@@ -1598,11 +1592,6 @@
     <font>
       <sz val="10.000000"/>
       <color rgb="FFAC0000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="14.000000"/>
-      <color indexed="2"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -2028,7 +2017,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="109">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2288,10 +2277,7 @@
     <xf fontId="16" fillId="9" borderId="13" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf fontId="22" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="23" fillId="7" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="22" fillId="7" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf fontId="2" fillId="7" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3508,8 +3494,8 @@
     <col customWidth="1" min="1" max="1" style="1" width="15.81640625"/>
     <col customWidth="1" min="2" max="2" style="1" width="74.08984375"/>
     <col customWidth="1" min="3" max="3" style="1" width="34"/>
-    <col customWidth="1" min="4" max="25" style="1" width="10.08984375"/>
-    <col min="26" max="16384" style="1" width="14.453125"/>
+    <col customWidth="1" min="4" max="22" style="1" width="10.08984375"/>
+    <col min="23" max="16384" style="1" width="14.453125"/>
   </cols>
   <sheetData>
     <row r="1" ht="39" customHeight="1">
@@ -3537,9 +3523,6 @@
       <c r="T1" s="5"/>
       <c r="U1" s="5"/>
       <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
-      <c r="X1" s="5"/>
-      <c r="Y1" s="5"/>
     </row>
     <row r="2" ht="24.75" customHeight="1">
       <c r="A2" s="6" t="s">
@@ -3570,9 +3553,6 @@
       <c r="T2" s="7"/>
       <c r="U2" s="7"/>
       <c r="V2" s="7"/>
-      <c r="W2" s="7"/>
-      <c r="X2" s="7"/>
-      <c r="Y2" s="7"/>
     </row>
     <row r="3" s="8" customFormat="1" ht="24.75" customHeight="1">
       <c r="A3" s="9" t="s">
@@ -3601,9 +3581,6 @@
       <c r="T3" s="12"/>
       <c r="U3" s="12"/>
       <c r="V3" s="12"/>
-      <c r="W3" s="12"/>
-      <c r="X3" s="12"/>
-      <c r="Y3" s="12"/>
     </row>
     <row r="4" ht="92.400000000000006" customHeight="1">
       <c r="A4" s="13">
@@ -3634,9 +3611,6 @@
       <c r="T4" s="15"/>
       <c r="U4" s="15"/>
       <c r="V4" s="15"/>
-      <c r="W4" s="15"/>
-      <c r="X4" s="15"/>
-      <c r="Y4" s="15"/>
     </row>
     <row r="5" ht="34.5" customHeight="1">
       <c r="A5" s="16" t="s">
@@ -3663,9 +3637,6 @@
       <c r="T5" s="19"/>
       <c r="U5" s="19"/>
       <c r="V5" s="19"/>
-      <c r="W5" s="19"/>
-      <c r="X5" s="19"/>
-      <c r="Y5" s="19"/>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="20" t="s">
@@ -3694,9 +3665,6 @@
       <c r="T6" s="15"/>
       <c r="U6" s="15"/>
       <c r="V6" s="15"/>
-      <c r="W6" s="15"/>
-      <c r="X6" s="15"/>
-      <c r="Y6" s="15"/>
     </row>
     <row r="7" ht="27.75" customHeight="1">
       <c r="A7" s="23" t="s">
@@ -3727,9 +3695,6 @@
       <c r="T7" s="15"/>
       <c r="U7" s="15"/>
       <c r="V7" s="15"/>
-      <c r="W7" s="15"/>
-      <c r="X7" s="15"/>
-      <c r="Y7" s="15"/>
     </row>
     <row r="8" ht="27.75" customHeight="1">
       <c r="A8" s="25" t="s">
@@ -3760,9 +3725,6 @@
       <c r="T8" s="15"/>
       <c r="U8" s="15"/>
       <c r="V8" s="15"/>
-      <c r="W8" s="15"/>
-      <c r="X8" s="15"/>
-      <c r="Y8" s="15"/>
     </row>
     <row r="9" ht="27.75" customHeight="1">
       <c r="A9" s="25" t="s">
@@ -3793,9 +3755,6 @@
       <c r="T9" s="15"/>
       <c r="U9" s="15"/>
       <c r="V9" s="15"/>
-      <c r="W9" s="15"/>
-      <c r="X9" s="15"/>
-      <c r="Y9" s="15"/>
     </row>
     <row r="10" ht="27.75" customHeight="1">
       <c r="A10" s="25" t="s">
@@ -3824,9 +3783,6 @@
       <c r="T10" s="15"/>
       <c r="U10" s="15"/>
       <c r="V10" s="15"/>
-      <c r="W10" s="15"/>
-      <c r="X10" s="15"/>
-      <c r="Y10" s="15"/>
     </row>
     <row r="11" ht="27.75" customHeight="1">
       <c r="A11" s="27" t="s">
@@ -3855,9 +3811,6 @@
       <c r="T11" s="30"/>
       <c r="U11" s="30"/>
       <c r="V11" s="30"/>
-      <c r="W11" s="30"/>
-      <c r="X11" s="30"/>
-      <c r="Y11" s="30"/>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="31" t="s">
@@ -3886,9 +3839,6 @@
       <c r="T12" s="30"/>
       <c r="U12" s="30"/>
       <c r="V12" s="30"/>
-      <c r="W12" s="30"/>
-      <c r="X12" s="30"/>
-      <c r="Y12" s="30"/>
     </row>
     <row r="13" ht="27.75" customHeight="1">
       <c r="A13" s="34" t="s">
@@ -3919,9 +3869,6 @@
       <c r="T13" s="30"/>
       <c r="U13" s="30"/>
       <c r="V13" s="30"/>
-      <c r="W13" s="30"/>
-      <c r="X13" s="30"/>
-      <c r="Y13" s="30"/>
     </row>
     <row r="14" ht="27.75" customHeight="1">
       <c r="A14" s="35" t="s">
@@ -3952,9 +3899,6 @@
       <c r="T14" s="30"/>
       <c r="U14" s="30"/>
       <c r="V14" s="30"/>
-      <c r="W14" s="30"/>
-      <c r="X14" s="30"/>
-      <c r="Y14" s="30"/>
     </row>
     <row r="15" ht="27.75" customHeight="1">
       <c r="A15" s="35" t="s">
@@ -3985,9 +3929,6 @@
       <c r="T15" s="30"/>
       <c r="U15" s="30"/>
       <c r="V15" s="30"/>
-      <c r="W15" s="30"/>
-      <c r="X15" s="30"/>
-      <c r="Y15" s="30"/>
     </row>
     <row r="16" ht="27.75" customHeight="1">
       <c r="A16" s="35" t="s">
@@ -4018,9 +3959,6 @@
       <c r="T16" s="30"/>
       <c r="U16" s="30"/>
       <c r="V16" s="30"/>
-      <c r="W16" s="30"/>
-      <c r="X16" s="30"/>
-      <c r="Y16" s="30"/>
     </row>
     <row r="17" ht="27.75" customHeight="1">
       <c r="A17" s="14" t="s">
@@ -4051,9 +3989,6 @@
       <c r="T17" s="30"/>
       <c r="U17" s="30"/>
       <c r="V17" s="30"/>
-      <c r="W17" s="30"/>
-      <c r="X17" s="30"/>
-      <c r="Y17" s="30"/>
     </row>
     <row r="18" ht="27.75" customHeight="1">
       <c r="A18" s="35" t="s">
@@ -4082,9 +4017,6 @@
       <c r="T18" s="30"/>
       <c r="U18" s="30"/>
       <c r="V18" s="30"/>
-      <c r="W18" s="30"/>
-      <c r="X18" s="30"/>
-      <c r="Y18" s="30"/>
     </row>
     <row r="19" ht="22.75" customHeight="1">
       <c r="A19" s="36" t="s">
@@ -4115,9 +4047,6 @@
       <c r="T19" s="30"/>
       <c r="U19" s="30"/>
       <c r="V19" s="30"/>
-      <c r="W19" s="30"/>
-      <c r="X19" s="30"/>
-      <c r="Y19" s="30"/>
     </row>
     <row r="20" ht="27.75" customHeight="1">
       <c r="A20" s="37"/>
@@ -4146,9 +4075,6 @@
       <c r="T20" s="30"/>
       <c r="U20" s="30"/>
       <c r="V20" s="30"/>
-      <c r="W20" s="30"/>
-      <c r="X20" s="30"/>
-      <c r="Y20" s="30"/>
     </row>
     <row r="21" ht="38.25" customHeight="1">
       <c r="A21" s="38" t="s">
@@ -4177,9 +4103,6 @@
       <c r="T21" s="30"/>
       <c r="U21" s="30"/>
       <c r="V21" s="30"/>
-      <c r="W21" s="30"/>
-      <c r="X21" s="30"/>
-      <c r="Y21" s="30"/>
     </row>
     <row r="22" ht="235.25" customHeight="1">
       <c r="A22" s="40" t="s">
@@ -4210,9 +4133,6 @@
       <c r="T22" s="30"/>
       <c r="U22" s="30"/>
       <c r="V22" s="30"/>
-      <c r="W22" s="30"/>
-      <c r="X22" s="30"/>
-      <c r="Y22" s="30"/>
     </row>
     <row r="23" ht="27.75" customHeight="1">
       <c r="A23" s="43" t="s">
@@ -4241,9 +4161,6 @@
       <c r="T23" s="15"/>
       <c r="U23" s="15"/>
       <c r="V23" s="15"/>
-      <c r="W23" s="15"/>
-      <c r="X23" s="15"/>
-      <c r="Y23" s="15"/>
     </row>
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="31" t="s">
@@ -4272,9 +4189,6 @@
       <c r="T24" s="15"/>
       <c r="U24" s="15"/>
       <c r="V24" s="15"/>
-      <c r="W24" s="15"/>
-      <c r="X24" s="15"/>
-      <c r="Y24" s="15"/>
     </row>
     <row r="25" ht="27.75" customHeight="1">
       <c r="A25" s="34" t="s">
@@ -4305,9 +4219,6 @@
       <c r="T25" s="15"/>
       <c r="U25" s="15"/>
       <c r="V25" s="15"/>
-      <c r="W25" s="15"/>
-      <c r="X25" s="15"/>
-      <c r="Y25" s="15"/>
     </row>
     <row r="26" ht="27.75" customHeight="1">
       <c r="A26" s="34" t="s">
@@ -4338,9 +4249,6 @@
       <c r="T26" s="15"/>
       <c r="U26" s="15"/>
       <c r="V26" s="15"/>
-      <c r="W26" s="15"/>
-      <c r="X26" s="15"/>
-      <c r="Y26" s="15"/>
     </row>
     <row r="27" ht="27.75" customHeight="1">
       <c r="A27" s="34" t="s">
@@ -4371,9 +4279,6 @@
       <c r="T27" s="30"/>
       <c r="U27" s="30"/>
       <c r="V27" s="30"/>
-      <c r="W27" s="30"/>
-      <c r="X27" s="30"/>
-      <c r="Y27" s="30"/>
     </row>
     <row r="28" ht="27.75" customHeight="1">
       <c r="A28" s="14" t="s">
@@ -4404,9 +4309,6 @@
       <c r="T28" s="30"/>
       <c r="U28" s="30"/>
       <c r="V28" s="30"/>
-      <c r="W28" s="30"/>
-      <c r="X28" s="30"/>
-      <c r="Y28" s="30"/>
     </row>
     <row r="29" ht="27.75" customHeight="1">
       <c r="A29" s="14" t="s">
@@ -4435,9 +4337,6 @@
       <c r="T29" s="30"/>
       <c r="U29" s="30"/>
       <c r="V29" s="30"/>
-      <c r="W29" s="30"/>
-      <c r="X29" s="30"/>
-      <c r="Y29" s="30"/>
     </row>
     <row r="30" ht="27.75" customHeight="1">
       <c r="A30" s="14" t="s">
@@ -4466,9 +4365,6 @@
       <c r="T30" s="30"/>
       <c r="U30" s="30"/>
       <c r="V30" s="30"/>
-      <c r="W30" s="30"/>
-      <c r="X30" s="30"/>
-      <c r="Y30" s="30"/>
     </row>
     <row r="31" ht="27.75" customHeight="1">
       <c r="A31" s="14" t="s">
@@ -4499,9 +4395,6 @@
       <c r="T31" s="15"/>
       <c r="U31" s="15"/>
       <c r="V31" s="15"/>
-      <c r="W31" s="15"/>
-      <c r="X31" s="15"/>
-      <c r="Y31" s="15"/>
     </row>
     <row r="32" ht="27.75" customHeight="1">
       <c r="A32" s="14" t="s">
@@ -4532,9 +4425,6 @@
       <c r="T32" s="15"/>
       <c r="U32" s="15"/>
       <c r="V32" s="15"/>
-      <c r="W32" s="15"/>
-      <c r="X32" s="15"/>
-      <c r="Y32" s="15"/>
     </row>
     <row r="33" ht="117.65000000000001" customHeight="1">
       <c r="A33" s="46" t="s">
@@ -4565,9 +4455,6 @@
       <c r="T33" s="15"/>
       <c r="U33" s="15"/>
       <c r="V33" s="15"/>
-      <c r="W33" s="15"/>
-      <c r="X33" s="15"/>
-      <c r="Y33" s="15"/>
     </row>
     <row r="34" ht="22.5" customHeight="1">
       <c r="A34" s="49">
@@ -4596,9 +4483,6 @@
       <c r="T34" s="15"/>
       <c r="U34" s="15"/>
       <c r="V34" s="15"/>
-      <c r="W34" s="15"/>
-      <c r="X34" s="15"/>
-      <c r="Y34" s="15"/>
     </row>
     <row r="35" ht="39" customHeight="1">
       <c r="A35" s="2" t="s">
@@ -4625,9 +4509,6 @@
       <c r="T35" s="19"/>
       <c r="U35" s="19"/>
       <c r="V35" s="19"/>
-      <c r="W35" s="19"/>
-      <c r="X35" s="19"/>
-      <c r="Y35" s="19"/>
     </row>
     <row r="36" ht="24.75" customHeight="1">
       <c r="A36" s="6" t="s">
@@ -4658,9 +4539,6 @@
       <c r="T36" s="7"/>
       <c r="U36" s="7"/>
       <c r="V36" s="7"/>
-      <c r="W36" s="7"/>
-      <c r="X36" s="7"/>
-      <c r="Y36" s="7"/>
     </row>
     <row r="37" ht="34.5" customHeight="1">
       <c r="A37" s="53" t="s">
@@ -4687,9 +4565,6 @@
       <c r="T37" s="15"/>
       <c r="U37" s="15"/>
       <c r="V37" s="15"/>
-      <c r="W37" s="15"/>
-      <c r="X37" s="15"/>
-      <c r="Y37" s="15"/>
     </row>
     <row r="38" ht="29.25" customHeight="1">
       <c r="A38" s="56" t="s">
@@ -4718,9 +4593,6 @@
       <c r="T38" s="15"/>
       <c r="U38" s="15"/>
       <c r="V38" s="15"/>
-      <c r="W38" s="15"/>
-      <c r="X38" s="15"/>
-      <c r="Y38" s="15"/>
     </row>
     <row r="39" ht="28.5" customHeight="1">
       <c r="A39" s="14" t="s">
@@ -4751,9 +4623,6 @@
       <c r="T39" s="15"/>
       <c r="U39" s="15"/>
       <c r="V39" s="15"/>
-      <c r="W39" s="15"/>
-      <c r="X39" s="15"/>
-      <c r="Y39" s="15"/>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="14" t="s">
@@ -4784,9 +4653,6 @@
       <c r="T40" s="15"/>
       <c r="U40" s="15"/>
       <c r="V40" s="15"/>
-      <c r="W40" s="15"/>
-      <c r="X40" s="15"/>
-      <c r="Y40" s="15"/>
     </row>
     <row r="41" ht="30.75" customHeight="1">
       <c r="A41" s="14" t="s">
@@ -4817,9 +4683,6 @@
       <c r="T41" s="15"/>
       <c r="U41" s="15"/>
       <c r="V41" s="15"/>
-      <c r="W41" s="15"/>
-      <c r="X41" s="15"/>
-      <c r="Y41" s="15"/>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="14" t="s">
@@ -4850,9 +4713,6 @@
       <c r="T42" s="15"/>
       <c r="U42" s="15"/>
       <c r="V42" s="15"/>
-      <c r="W42" s="15"/>
-      <c r="X42" s="15"/>
-      <c r="Y42" s="15"/>
     </row>
     <row r="43" ht="27" customHeight="1">
       <c r="A43" s="14" t="s">
@@ -4883,9 +4743,6 @@
       <c r="T43" s="15"/>
       <c r="U43" s="15"/>
       <c r="V43" s="15"/>
-      <c r="W43" s="15"/>
-      <c r="X43" s="15"/>
-      <c r="Y43" s="15"/>
     </row>
     <row r="44" ht="27.75" customHeight="1">
       <c r="A44" s="56" t="s">
@@ -4914,9 +4771,6 @@
       <c r="T44" s="15"/>
       <c r="U44" s="15"/>
       <c r="V44" s="15"/>
-      <c r="W44" s="15"/>
-      <c r="X44" s="15"/>
-      <c r="Y44" s="15"/>
     </row>
     <row r="45" ht="42" customHeight="1">
       <c r="A45" s="58" t="s">
@@ -4945,9 +4799,6 @@
       <c r="T45" s="15"/>
       <c r="U45" s="15"/>
       <c r="V45" s="15"/>
-      <c r="W45" s="15"/>
-      <c r="X45" s="15"/>
-      <c r="Y45" s="15"/>
     </row>
     <row r="46" ht="42" customHeight="1">
       <c r="A46" s="61" t="s">
@@ -4976,9 +4827,6 @@
       <c r="T46" s="15"/>
       <c r="U46" s="15"/>
       <c r="V46" s="15"/>
-      <c r="W46" s="15"/>
-      <c r="X46" s="15"/>
-      <c r="Y46" s="15"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="64"/>
@@ -5007,9 +4855,6 @@
       <c r="T47" s="15"/>
       <c r="U47" s="15"/>
       <c r="V47" s="15"/>
-      <c r="W47" s="15"/>
-      <c r="X47" s="15"/>
-      <c r="Y47" s="15"/>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="64"/>
@@ -5038,9 +4883,6 @@
       <c r="T48" s="15"/>
       <c r="U48" s="15"/>
       <c r="V48" s="15"/>
-      <c r="W48" s="15"/>
-      <c r="X48" s="15"/>
-      <c r="Y48" s="15"/>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="65" t="s">
@@ -5071,9 +4913,6 @@
       <c r="T49" s="15"/>
       <c r="U49" s="15"/>
       <c r="V49" s="15"/>
-      <c r="W49" s="15"/>
-      <c r="X49" s="15"/>
-      <c r="Y49" s="15"/>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="65" t="s">
@@ -5104,9 +4943,6 @@
       <c r="T50" s="15"/>
       <c r="U50" s="15"/>
       <c r="V50" s="15"/>
-      <c r="W50" s="15"/>
-      <c r="X50" s="15"/>
-      <c r="Y50" s="15"/>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="65" t="s">
@@ -5135,9 +4971,6 @@
       <c r="T51" s="15"/>
       <c r="U51" s="15"/>
       <c r="V51" s="15"/>
-      <c r="W51" s="15"/>
-      <c r="X51" s="15"/>
-      <c r="Y51" s="15"/>
     </row>
     <row r="52" ht="27.75" customHeight="1">
       <c r="A52" s="56" t="s">
@@ -5166,9 +4999,6 @@
       <c r="T52" s="67"/>
       <c r="U52" s="67"/>
       <c r="V52" s="67"/>
-      <c r="W52" s="67"/>
-      <c r="X52" s="67"/>
-      <c r="Y52" s="67"/>
     </row>
     <row r="53" ht="28.5" customHeight="1">
       <c r="A53" s="68" t="s">
@@ -5197,9 +5027,6 @@
       <c r="T53" s="15"/>
       <c r="U53" s="15"/>
       <c r="V53" s="15"/>
-      <c r="W53" s="15"/>
-      <c r="X53" s="15"/>
-      <c r="Y53" s="15"/>
     </row>
     <row r="54" ht="27.75" customHeight="1">
       <c r="A54" s="38" t="s">
@@ -5228,9 +5055,6 @@
       <c r="T54" s="15"/>
       <c r="U54" s="15"/>
       <c r="V54" s="15"/>
-      <c r="W54" s="15"/>
-      <c r="X54" s="15"/>
-      <c r="Y54" s="15"/>
     </row>
     <row r="55" ht="27.75" customHeight="1">
       <c r="A55" s="34" t="s">
@@ -5261,9 +5085,6 @@
       <c r="T55" s="70"/>
       <c r="U55" s="70"/>
       <c r="V55" s="70"/>
-      <c r="W55" s="70"/>
-      <c r="X55" s="70"/>
-      <c r="Y55" s="70"/>
     </row>
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="71" t="s">
@@ -5292,9 +5113,6 @@
       <c r="T56" s="70"/>
       <c r="U56" s="70"/>
       <c r="V56" s="70"/>
-      <c r="W56" s="70"/>
-      <c r="X56" s="70"/>
-      <c r="Y56" s="70"/>
     </row>
     <row r="57" ht="26.25" customHeight="1">
       <c r="A57" s="73" t="s">
@@ -5325,9 +5143,6 @@
       <c r="T57" s="70"/>
       <c r="U57" s="70"/>
       <c r="V57" s="70"/>
-      <c r="W57" s="70"/>
-      <c r="X57" s="70"/>
-      <c r="Y57" s="70"/>
     </row>
     <row r="58" ht="27.75" customHeight="1">
       <c r="A58" s="65" t="s">
@@ -5358,9 +5173,6 @@
       <c r="T58" s="70"/>
       <c r="U58" s="70"/>
       <c r="V58" s="70"/>
-      <c r="W58" s="70"/>
-      <c r="X58" s="70"/>
-      <c r="Y58" s="70"/>
     </row>
     <row r="59" ht="27.75" customHeight="1">
       <c r="A59" s="73" t="s">
@@ -5372,6 +5184,7 @@
       <c r="C59" s="65" t="s">
         <v>127</v>
       </c>
+      <c r="D59" s="70"/>
       <c r="E59" s="70"/>
       <c r="F59" s="70"/>
       <c r="G59" s="70"/>
@@ -5390,9 +5203,6 @@
       <c r="T59" s="70"/>
       <c r="U59" s="70"/>
       <c r="V59" s="70"/>
-      <c r="W59" s="70"/>
-      <c r="X59" s="70"/>
-      <c r="Y59" s="70"/>
     </row>
     <row r="60" ht="27.75" customHeight="1">
       <c r="A60" s="65" t="s">
@@ -5423,9 +5233,6 @@
       <c r="T60" s="70"/>
       <c r="U60" s="70"/>
       <c r="V60" s="70"/>
-      <c r="W60" s="70"/>
-      <c r="X60" s="70"/>
-      <c r="Y60" s="70"/>
     </row>
     <row r="61" ht="27.75" customHeight="1">
       <c r="A61" s="65" t="s">
@@ -5456,9 +5263,6 @@
       <c r="T61" s="70"/>
       <c r="U61" s="70"/>
       <c r="V61" s="70"/>
-      <c r="W61" s="70"/>
-      <c r="X61" s="70"/>
-      <c r="Y61" s="70"/>
     </row>
     <row r="62" ht="27.75" customHeight="1">
       <c r="A62" s="65" t="s">
@@ -5487,9 +5291,6 @@
       <c r="T62" s="70"/>
       <c r="U62" s="70"/>
       <c r="V62" s="70"/>
-      <c r="W62" s="70"/>
-      <c r="X62" s="70"/>
-      <c r="Y62" s="70"/>
     </row>
     <row r="63" ht="46.75" customHeight="1">
       <c r="A63" s="75" t="s">
@@ -5518,9 +5319,6 @@
       <c r="T63" s="70"/>
       <c r="U63" s="70"/>
       <c r="V63" s="70"/>
-      <c r="W63" s="70"/>
-      <c r="X63" s="70"/>
-      <c r="Y63" s="70"/>
     </row>
     <row r="64" ht="27.75" customHeight="1">
       <c r="A64" s="64"/>
@@ -5549,9 +5347,6 @@
       <c r="T64" s="70"/>
       <c r="U64" s="70"/>
       <c r="V64" s="70"/>
-      <c r="W64" s="70"/>
-      <c r="X64" s="70"/>
-      <c r="Y64" s="70"/>
     </row>
     <row r="65" ht="27.75" customHeight="1">
       <c r="A65" s="64"/>
@@ -5580,9 +5375,6 @@
       <c r="T65" s="70"/>
       <c r="U65" s="70"/>
       <c r="V65" s="70"/>
-      <c r="W65" s="70"/>
-      <c r="X65" s="70"/>
-      <c r="Y65" s="70"/>
     </row>
     <row r="66" ht="27.75" customHeight="1">
       <c r="A66" s="78"/>
@@ -5611,9 +5403,6 @@
       <c r="T66" s="70"/>
       <c r="U66" s="70"/>
       <c r="V66" s="70"/>
-      <c r="W66" s="70"/>
-      <c r="X66" s="70"/>
-      <c r="Y66" s="70"/>
     </row>
     <row r="67" ht="27.649999999999999" customHeight="1">
       <c r="A67" s="34">
@@ -5642,9 +5431,6 @@
       <c r="T67" s="70"/>
       <c r="U67" s="70"/>
       <c r="V67" s="70"/>
-      <c r="W67" s="70"/>
-      <c r="X67" s="70"/>
-      <c r="Y67" s="70"/>
     </row>
     <row r="68" ht="10.75" customHeight="1">
       <c r="A68" s="79"/>
@@ -5669,9 +5455,6 @@
       <c r="T68" s="15"/>
       <c r="U68" s="15"/>
       <c r="V68" s="15"/>
-      <c r="W68" s="15"/>
-      <c r="X68" s="15"/>
-      <c r="Y68" s="15"/>
     </row>
     <row r="69" ht="39" customHeight="1">
       <c r="A69" s="2" t="s">
@@ -5698,9 +5481,6 @@
       <c r="T69" s="19"/>
       <c r="U69" s="19"/>
       <c r="V69" s="19"/>
-      <c r="W69" s="19"/>
-      <c r="X69" s="19"/>
-      <c r="Y69" s="19"/>
     </row>
     <row r="70" ht="27.75" customHeight="1">
       <c r="A70" s="6" t="s">
@@ -5731,9 +5511,6 @@
       <c r="T70" s="7"/>
       <c r="U70" s="7"/>
       <c r="V70" s="7"/>
-      <c r="W70" s="7"/>
-      <c r="X70" s="7"/>
-      <c r="Y70" s="7"/>
     </row>
     <row r="71" ht="34.5" customHeight="1">
       <c r="A71" s="16" t="s">
@@ -5760,9 +5537,6 @@
       <c r="T71" s="19"/>
       <c r="U71" s="19"/>
       <c r="V71" s="19"/>
-      <c r="W71" s="19"/>
-      <c r="X71" s="19"/>
-      <c r="Y71" s="19"/>
     </row>
     <row r="72" ht="185.40000000000001" customHeight="1">
       <c r="A72" s="81" t="s">
@@ -5793,9 +5567,6 @@
       <c r="T72" s="84"/>
       <c r="U72" s="84"/>
       <c r="V72" s="84"/>
-      <c r="W72" s="84"/>
-      <c r="X72" s="84"/>
-      <c r="Y72" s="84"/>
     </row>
     <row r="73" ht="27.75" customHeight="1">
       <c r="A73" s="38" t="s">
@@ -5824,9 +5595,6 @@
       <c r="T73" s="15"/>
       <c r="U73" s="15"/>
       <c r="V73" s="15"/>
-      <c r="W73" s="15"/>
-      <c r="X73" s="15"/>
-      <c r="Y73" s="15"/>
     </row>
     <row r="74" ht="42" customHeight="1">
       <c r="A74" s="85" t="s">
@@ -5836,7 +5604,9 @@
         <v>148</v>
       </c>
       <c r="C74" s="60"/>
-      <c r="D74" s="1"/>
+      <c r="D74" s="15"/>
+      <c r="E74" s="15"/>
+      <c r="F74" s="15"/>
       <c r="G74" s="15"/>
       <c r="H74" s="15"/>
       <c r="I74" s="15"/>
@@ -5853,9 +5623,6 @@
       <c r="T74" s="15"/>
       <c r="U74" s="15"/>
       <c r="V74" s="15"/>
-      <c r="W74" s="15"/>
-      <c r="X74" s="15"/>
-      <c r="Y74" s="15"/>
     </row>
     <row r="75" ht="27.75" customHeight="1">
       <c r="A75" s="14" t="s">
@@ -5867,9 +5634,9 @@
       <c r="C75" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="D75" s="87"/>
-      <c r="E75" s="87"/>
-      <c r="F75" s="87"/>
+      <c r="D75" s="19"/>
+      <c r="E75" s="19"/>
+      <c r="F75" s="19"/>
       <c r="G75" s="19"/>
       <c r="H75" s="19"/>
       <c r="I75" s="19"/>
@@ -5886,9 +5653,6 @@
       <c r="T75" s="19"/>
       <c r="U75" s="19"/>
       <c r="V75" s="19"/>
-      <c r="W75" s="19"/>
-      <c r="X75" s="19"/>
-      <c r="Y75" s="19"/>
     </row>
     <row r="76" ht="27.75" customHeight="1">
       <c r="A76" s="14" t="s">
@@ -5900,9 +5664,9 @@
       <c r="C76" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="D76" s="87"/>
-      <c r="E76" s="87"/>
-      <c r="F76" s="87"/>
+      <c r="D76" s="19"/>
+      <c r="E76" s="19"/>
+      <c r="F76" s="19"/>
       <c r="G76" s="19"/>
       <c r="H76" s="19"/>
       <c r="I76" s="19"/>
@@ -5919,9 +5683,6 @@
       <c r="T76" s="19"/>
       <c r="U76" s="19"/>
       <c r="V76" s="19"/>
-      <c r="W76" s="19"/>
-      <c r="X76" s="19"/>
-      <c r="Y76" s="19"/>
     </row>
     <row r="77" ht="27.75" customHeight="1">
       <c r="A77" s="14" t="s">
@@ -5952,9 +5713,6 @@
       <c r="T77" s="19"/>
       <c r="U77" s="19"/>
       <c r="V77" s="19"/>
-      <c r="W77" s="19"/>
-      <c r="X77" s="19"/>
-      <c r="Y77" s="19"/>
     </row>
     <row r="78" ht="27.75" customHeight="1">
       <c r="A78" s="14" t="s">
@@ -5985,15 +5743,12 @@
       <c r="T78" s="19"/>
       <c r="U78" s="19"/>
       <c r="V78" s="19"/>
-      <c r="W78" s="19"/>
-      <c r="X78" s="19"/>
-      <c r="Y78" s="19"/>
     </row>
     <row r="79" ht="27.75" customHeight="1">
       <c r="A79" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="B79" s="88" t="s">
+      <c r="B79" s="87" t="s">
         <v>21</v>
       </c>
       <c r="C79" s="14"/>
@@ -6016,9 +5771,6 @@
       <c r="T79" s="19"/>
       <c r="U79" s="19"/>
       <c r="V79" s="19"/>
-      <c r="W79" s="19"/>
-      <c r="X79" s="19"/>
-      <c r="Y79" s="19"/>
     </row>
     <row r="80" ht="31.5" customHeight="1">
       <c r="A80" s="14" t="s">
@@ -6027,7 +5779,7 @@
       <c r="B80" s="39" t="s">
         <v>161</v>
       </c>
-      <c r="C80" s="89"/>
+      <c r="C80" s="88"/>
       <c r="D80" s="15"/>
       <c r="E80" s="15"/>
       <c r="F80" s="15"/>
@@ -6047,9 +5799,6 @@
       <c r="T80" s="15"/>
       <c r="U80" s="15"/>
       <c r="V80" s="15"/>
-      <c r="W80" s="15"/>
-      <c r="X80" s="15"/>
-      <c r="Y80" s="15"/>
     </row>
     <row r="81" ht="27.75" customHeight="1">
       <c r="A81" s="14" t="s">
@@ -6080,9 +5829,6 @@
       <c r="T81" s="19"/>
       <c r="U81" s="19"/>
       <c r="V81" s="19"/>
-      <c r="W81" s="19"/>
-      <c r="X81" s="19"/>
-      <c r="Y81" s="19"/>
     </row>
     <row r="82" ht="27.75" customHeight="1">
       <c r="A82" s="14" t="s">
@@ -6113,9 +5859,6 @@
       <c r="T82" s="19"/>
       <c r="U82" s="19"/>
       <c r="V82" s="19"/>
-      <c r="W82" s="19"/>
-      <c r="X82" s="19"/>
-      <c r="Y82" s="19"/>
     </row>
     <row r="83" ht="27.75" customHeight="1">
       <c r="A83" s="14" t="s">
@@ -6146,40 +5889,34 @@
       <c r="T83" s="19"/>
       <c r="U83" s="19"/>
       <c r="V83" s="19"/>
-      <c r="W83" s="19"/>
-      <c r="X83" s="19"/>
-      <c r="Y83" s="19"/>
     </row>
     <row r="84" ht="32.399999999999999" customHeight="1">
-      <c r="A84" s="90" t="s">
+      <c r="A84" s="89" t="s">
         <v>170</v>
       </c>
-      <c r="B84" s="91" t="s">
+      <c r="B84" s="90" t="s">
         <v>171</v>
       </c>
-      <c r="C84" s="92"/>
-      <c r="D84" s="93"/>
-      <c r="E84" s="93"/>
-      <c r="F84" s="93"/>
-      <c r="G84" s="93"/>
-      <c r="H84" s="93"/>
-      <c r="I84" s="93"/>
-      <c r="J84" s="93"/>
-      <c r="K84" s="93"/>
-      <c r="L84" s="93"/>
-      <c r="M84" s="93"/>
-      <c r="N84" s="93"/>
-      <c r="O84" s="93"/>
-      <c r="P84" s="93"/>
-      <c r="Q84" s="93"/>
-      <c r="R84" s="93"/>
-      <c r="S84" s="93"/>
-      <c r="T84" s="93"/>
-      <c r="U84" s="93"/>
-      <c r="V84" s="93"/>
-      <c r="W84" s="93"/>
-      <c r="X84" s="93"/>
-      <c r="Y84" s="93"/>
+      <c r="C84" s="91"/>
+      <c r="D84" s="92"/>
+      <c r="E84" s="92"/>
+      <c r="F84" s="92"/>
+      <c r="G84" s="92"/>
+      <c r="H84" s="92"/>
+      <c r="I84" s="92"/>
+      <c r="J84" s="92"/>
+      <c r="K84" s="92"/>
+      <c r="L84" s="92"/>
+      <c r="M84" s="92"/>
+      <c r="N84" s="92"/>
+      <c r="O84" s="92"/>
+      <c r="P84" s="92"/>
+      <c r="Q84" s="92"/>
+      <c r="R84" s="92"/>
+      <c r="S84" s="92"/>
+      <c r="T84" s="92"/>
+      <c r="U84" s="92"/>
+      <c r="V84" s="92"/>
     </row>
     <row r="85" ht="27.75" customHeight="1">
       <c r="A85" s="35" t="s">
@@ -6208,12 +5945,9 @@
       <c r="T85" s="19"/>
       <c r="U85" s="19"/>
       <c r="V85" s="19"/>
-      <c r="W85" s="19"/>
-      <c r="X85" s="19"/>
-      <c r="Y85" s="19"/>
     </row>
     <row r="86" ht="27.75" customHeight="1">
-      <c r="A86" s="94" t="s">
+      <c r="A86" s="93" t="s">
         <v>174</v>
       </c>
       <c r="B86" s="35" t="s">
@@ -6241,15 +5975,12 @@
       <c r="T86" s="19"/>
       <c r="U86" s="19"/>
       <c r="V86" s="19"/>
-      <c r="W86" s="19"/>
-      <c r="X86" s="19"/>
-      <c r="Y86" s="19"/>
     </row>
     <row r="87" ht="27.75" customHeight="1">
-      <c r="A87" s="94" t="s">
+      <c r="A87" s="93" t="s">
         <v>177</v>
       </c>
-      <c r="B87" s="95" t="s">
+      <c r="B87" s="94" t="s">
         <v>178</v>
       </c>
       <c r="C87" s="14" t="s">
@@ -6274,9 +6005,6 @@
       <c r="T87" s="19"/>
       <c r="U87" s="19"/>
       <c r="V87" s="19"/>
-      <c r="W87" s="19"/>
-      <c r="X87" s="19"/>
-      <c r="Y87" s="19"/>
     </row>
     <row r="88" ht="42" customHeight="1">
       <c r="A88" s="31" t="s">
@@ -6305,12 +6033,9 @@
       <c r="T88" s="15"/>
       <c r="U88" s="15"/>
       <c r="V88" s="15"/>
-      <c r="W88" s="15"/>
-      <c r="X88" s="15"/>
-      <c r="Y88" s="15"/>
     </row>
     <row r="89" ht="27.75" customHeight="1">
-      <c r="A89" s="96" t="s">
+      <c r="A89" s="95" t="s">
         <v>182</v>
       </c>
       <c r="B89" s="44" t="s">
@@ -6336,9 +6061,6 @@
       <c r="T89" s="19"/>
       <c r="U89" s="19"/>
       <c r="V89" s="19"/>
-      <c r="W89" s="19"/>
-      <c r="X89" s="19"/>
-      <c r="Y89" s="19"/>
     </row>
     <row r="90" ht="27.75" customHeight="1">
       <c r="A90" s="64"/>
@@ -6367,9 +6089,6 @@
       <c r="T90" s="19"/>
       <c r="U90" s="19"/>
       <c r="V90" s="19"/>
-      <c r="W90" s="19"/>
-      <c r="X90" s="19"/>
-      <c r="Y90" s="19"/>
     </row>
     <row r="91" ht="27.75" customHeight="1">
       <c r="A91" s="64"/>
@@ -6398,9 +6117,6 @@
       <c r="T91" s="19"/>
       <c r="U91" s="19"/>
       <c r="V91" s="19"/>
-      <c r="W91" s="19"/>
-      <c r="X91" s="19"/>
-      <c r="Y91" s="19"/>
     </row>
     <row r="92" ht="27.75" customHeight="1">
       <c r="A92" s="78"/>
@@ -6429,9 +6145,6 @@
       <c r="T92" s="19"/>
       <c r="U92" s="19"/>
       <c r="V92" s="19"/>
-      <c r="W92" s="19"/>
-      <c r="X92" s="19"/>
-      <c r="Y92" s="19"/>
     </row>
     <row r="93" ht="27.75" customHeight="1">
       <c r="A93" s="34" t="s">
@@ -6462,9 +6175,6 @@
       <c r="T93" s="19"/>
       <c r="U93" s="19"/>
       <c r="V93" s="19"/>
-      <c r="W93" s="19"/>
-      <c r="X93" s="19"/>
-      <c r="Y93" s="19"/>
     </row>
     <row r="94" ht="27.75" customHeight="1">
       <c r="A94" s="34" t="s">
@@ -6493,15 +6203,12 @@
       <c r="T94" s="19"/>
       <c r="U94" s="19"/>
       <c r="V94" s="19"/>
-      <c r="W94" s="19"/>
-      <c r="X94" s="19"/>
-      <c r="Y94" s="19"/>
     </row>
     <row r="95" ht="27.75" customHeight="1">
       <c r="A95" s="38" t="s">
         <v>194</v>
       </c>
-      <c r="B95" s="97" t="s">
+      <c r="B95" s="96" t="s">
         <v>195</v>
       </c>
       <c r="C95" s="33"/>
@@ -6524,15 +6231,12 @@
       <c r="T95" s="19"/>
       <c r="U95" s="19"/>
       <c r="V95" s="19"/>
-      <c r="W95" s="19"/>
-      <c r="X95" s="19"/>
-      <c r="Y95" s="19"/>
     </row>
     <row r="96" ht="232.25" customHeight="1">
-      <c r="A96" s="98" t="s">
+      <c r="A96" s="97" t="s">
         <v>196</v>
       </c>
-      <c r="B96" s="99" t="s">
+      <c r="B96" s="98" t="s">
         <v>197</v>
       </c>
       <c r="C96" s="83" t="s">
@@ -6557,9 +6261,6 @@
       <c r="T96" s="84"/>
       <c r="U96" s="84"/>
       <c r="V96" s="84"/>
-      <c r="W96" s="84"/>
-      <c r="X96" s="84"/>
-      <c r="Y96" s="84"/>
     </row>
     <row r="97" ht="27.75" customHeight="1">
       <c r="A97" s="34">
@@ -6588,15 +6289,12 @@
       <c r="T97" s="19"/>
       <c r="U97" s="19"/>
       <c r="V97" s="19"/>
-      <c r="W97" s="19"/>
-      <c r="X97" s="19"/>
-      <c r="Y97" s="19"/>
     </row>
     <row r="98" ht="29.25" customHeight="1">
-      <c r="A98" s="100">
+      <c r="A98" s="99">
         <v>0.6875</v>
       </c>
-      <c r="B98" s="101" t="s">
+      <c r="B98" s="100" t="s">
         <v>200</v>
       </c>
       <c r="C98" s="33"/>
@@ -6619,16 +6317,13 @@
       <c r="T98" s="19"/>
       <c r="U98" s="19"/>
       <c r="V98" s="19"/>
-      <c r="W98" s="19"/>
-      <c r="X98" s="19"/>
-      <c r="Y98" s="19"/>
     </row>
     <row r="99" ht="39" customHeight="1">
-      <c r="A99" s="102" t="s">
+      <c r="A99" s="101" t="s">
         <v>0</v>
       </c>
-      <c r="B99" s="103"/>
-      <c r="C99" s="104"/>
+      <c r="B99" s="102"/>
+      <c r="C99" s="103"/>
       <c r="D99" s="19"/>
       <c r="E99" s="19"/>
       <c r="F99" s="19"/>
@@ -6648,9 +6343,6 @@
       <c r="T99" s="19"/>
       <c r="U99" s="19"/>
       <c r="V99" s="19"/>
-      <c r="W99" s="19"/>
-      <c r="X99" s="19"/>
-      <c r="Y99" s="19"/>
     </row>
     <row r="100" ht="27.75" customHeight="1">
       <c r="A100" s="6" t="s">
@@ -6681,9 +6373,6 @@
       <c r="T100" s="7"/>
       <c r="U100" s="7"/>
       <c r="V100" s="7"/>
-      <c r="W100" s="7"/>
-      <c r="X100" s="7"/>
-      <c r="Y100" s="7"/>
     </row>
     <row r="101" ht="34.5" customHeight="1">
       <c r="A101" s="53" t="s">
@@ -6710,12 +6399,9 @@
       <c r="T101" s="15"/>
       <c r="U101" s="15"/>
       <c r="V101" s="15"/>
-      <c r="W101" s="15"/>
-      <c r="X101" s="15"/>
-      <c r="Y101" s="15"/>
     </row>
     <row r="102" ht="25.5" customHeight="1">
-      <c r="A102" s="105" t="s">
+      <c r="A102" s="104" t="s">
         <v>201</v>
       </c>
       <c r="B102" s="69" t="s">
@@ -6741,9 +6427,6 @@
       <c r="T102" s="84"/>
       <c r="U102" s="84"/>
       <c r="V102" s="84"/>
-      <c r="W102" s="84"/>
-      <c r="X102" s="84"/>
-      <c r="Y102" s="84"/>
     </row>
     <row r="103" ht="27.75" customHeight="1">
       <c r="A103" s="38" t="s">
@@ -6772,15 +6455,12 @@
       <c r="T103" s="15"/>
       <c r="U103" s="15"/>
       <c r="V103" s="15"/>
-      <c r="W103" s="15"/>
-      <c r="X103" s="15"/>
-      <c r="Y103" s="15"/>
     </row>
     <row r="104" ht="60" customHeight="1">
       <c r="A104" s="31" t="s">
         <v>203</v>
       </c>
-      <c r="B104" s="106" t="s">
+      <c r="B104" s="105" t="s">
         <v>204</v>
       </c>
       <c r="C104" s="33"/>
@@ -6803,12 +6483,9 @@
       <c r="T104" s="19"/>
       <c r="U104" s="19"/>
       <c r="V104" s="19"/>
-      <c r="W104" s="19"/>
-      <c r="X104" s="19"/>
-      <c r="Y104" s="19"/>
     </row>
     <row r="105" ht="27.75" customHeight="1">
-      <c r="A105" s="94" t="s">
+      <c r="A105" s="93" t="s">
         <v>205</v>
       </c>
       <c r="B105" s="35" t="s">
@@ -6836,12 +6513,9 @@
       <c r="T105" s="19"/>
       <c r="U105" s="19"/>
       <c r="V105" s="19"/>
-      <c r="W105" s="19"/>
-      <c r="X105" s="19"/>
-      <c r="Y105" s="19"/>
     </row>
     <row r="106" ht="27.75" customHeight="1">
-      <c r="A106" s="94" t="s">
+      <c r="A106" s="93" t="s">
         <v>32</v>
       </c>
       <c r="B106" s="35" t="s">
@@ -6869,9 +6543,6 @@
       <c r="T106" s="19"/>
       <c r="U106" s="19"/>
       <c r="V106" s="19"/>
-      <c r="W106" s="19"/>
-      <c r="X106" s="19"/>
-      <c r="Y106" s="19"/>
     </row>
     <row r="107" ht="27.75" customHeight="1">
       <c r="A107" s="34" t="s">
@@ -6900,9 +6571,6 @@
       <c r="T107" s="15"/>
       <c r="U107" s="15"/>
       <c r="V107" s="15"/>
-      <c r="W107" s="15"/>
-      <c r="X107" s="15"/>
-      <c r="Y107" s="15"/>
     </row>
     <row r="108" ht="27.75" customHeight="1">
       <c r="A108" s="14" t="s">
@@ -6911,7 +6579,7 @@
       <c r="B108" s="57" t="s">
         <v>213</v>
       </c>
-      <c r="C108" s="107"/>
+      <c r="C108" s="106"/>
       <c r="D108" s="19"/>
       <c r="E108" s="19"/>
       <c r="F108" s="19"/>
@@ -6931,9 +6599,6 @@
       <c r="T108" s="19"/>
       <c r="U108" s="19"/>
       <c r="V108" s="19"/>
-      <c r="W108" s="19"/>
-      <c r="X108" s="19"/>
-      <c r="Y108" s="19"/>
     </row>
     <row r="109" ht="27.75" customHeight="1">
       <c r="A109" s="34" t="s">
@@ -6964,9 +6629,6 @@
       <c r="T109" s="19"/>
       <c r="U109" s="19"/>
       <c r="V109" s="19"/>
-      <c r="W109" s="19"/>
-      <c r="X109" s="19"/>
-      <c r="Y109" s="19"/>
     </row>
     <row r="110" ht="27.75" customHeight="1">
       <c r="A110" s="34" t="s">
@@ -6997,15 +6659,12 @@
       <c r="T110" s="19"/>
       <c r="U110" s="19"/>
       <c r="V110" s="19"/>
-      <c r="W110" s="19"/>
-      <c r="X110" s="19"/>
-      <c r="Y110" s="19"/>
     </row>
     <row r="111" ht="42" customHeight="1">
       <c r="A111" s="31" t="s">
         <v>220</v>
       </c>
-      <c r="B111" s="106" t="s">
+      <c r="B111" s="105" t="s">
         <v>221</v>
       </c>
       <c r="C111" s="33"/>
@@ -7028,9 +6687,6 @@
       <c r="T111" s="19"/>
       <c r="U111" s="19"/>
       <c r="V111" s="19"/>
-      <c r="W111" s="19"/>
-      <c r="X111" s="19"/>
-      <c r="Y111" s="19"/>
     </row>
     <row r="112" ht="27.75" customHeight="1">
       <c r="A112" s="34" t="s">
@@ -7061,9 +6717,6 @@
       <c r="T112" s="19"/>
       <c r="U112" s="19"/>
       <c r="V112" s="19"/>
-      <c r="W112" s="19"/>
-      <c r="X112" s="19"/>
-      <c r="Y112" s="19"/>
     </row>
     <row r="113" ht="27.75" customHeight="1">
       <c r="A113" s="34" t="s">
@@ -7094,9 +6747,6 @@
       <c r="T113" s="19"/>
       <c r="U113" s="19"/>
       <c r="V113" s="19"/>
-      <c r="W113" s="19"/>
-      <c r="X113" s="19"/>
-      <c r="Y113" s="19"/>
     </row>
     <row r="114" ht="27.75" customHeight="1">
       <c r="A114" s="14" t="s">
@@ -7127,9 +6777,6 @@
       <c r="T114" s="19"/>
       <c r="U114" s="19"/>
       <c r="V114" s="19"/>
-      <c r="W114" s="19"/>
-      <c r="X114" s="19"/>
-      <c r="Y114" s="19"/>
     </row>
     <row r="115" ht="27.75" customHeight="1">
       <c r="A115" s="14" t="s">
@@ -7138,7 +6785,7 @@
       <c r="B115" s="35" t="s">
         <v>231</v>
       </c>
-      <c r="C115" s="108" t="s">
+      <c r="C115" s="107" t="s">
         <v>232</v>
       </c>
       <c r="D115" s="19"/>
@@ -7160,9 +6807,6 @@
       <c r="T115" s="19"/>
       <c r="U115" s="19"/>
       <c r="V115" s="19"/>
-      <c r="W115" s="19"/>
-      <c r="X115" s="19"/>
-      <c r="Y115" s="19"/>
     </row>
     <row r="116" ht="27.75" customHeight="1">
       <c r="A116" s="14" t="s">
@@ -7191,16 +6835,13 @@
       <c r="T116" s="19"/>
       <c r="U116" s="19"/>
       <c r="V116" s="19"/>
-      <c r="W116" s="19"/>
-      <c r="X116" s="19"/>
-      <c r="Y116" s="19"/>
     </row>
     <row r="117" ht="25.5" customHeight="1">
       <c r="A117" s="38" t="s">
-        <v>170</v>
+        <v>234</v>
       </c>
       <c r="B117" s="39" t="s">
-        <v>234</v>
+        <v>171</v>
       </c>
       <c r="C117" s="33"/>
       <c r="D117" s="19"/>
@@ -7222,18 +6863,15 @@
       <c r="T117" s="19"/>
       <c r="U117" s="19"/>
       <c r="V117" s="19"/>
-      <c r="W117" s="19"/>
-      <c r="X117" s="19"/>
-      <c r="Y117" s="19"/>
-    </row>
-    <row r="118" ht="28.5" customHeight="1">
-      <c r="A118" s="38" t="s">
+    </row>
+    <row r="118" ht="42" customHeight="1">
+      <c r="A118" s="31" t="s">
         <v>235</v>
       </c>
-      <c r="B118" s="39" t="s">
+      <c r="B118" s="105" t="s">
         <v>236</v>
       </c>
-      <c r="C118" s="89"/>
+      <c r="C118" s="33"/>
       <c r="D118" s="19"/>
       <c r="E118" s="19"/>
       <c r="F118" s="19"/>
@@ -7253,50 +6891,46 @@
       <c r="T118" s="19"/>
       <c r="U118" s="19"/>
       <c r="V118" s="19"/>
-      <c r="W118" s="19"/>
-      <c r="X118" s="19"/>
-      <c r="Y118" s="19"/>
-    </row>
-    <row r="119" ht="42" customHeight="1">
-      <c r="A119" s="31" t="s">
+    </row>
+    <row r="119" ht="27.75" customHeight="1">
+      <c r="A119" s="93" t="s">
         <v>237</v>
       </c>
-      <c r="B119" s="106" t="s">
+      <c r="B119" s="14" t="s">
         <v>238</v>
       </c>
-      <c r="C119" s="33"/>
-      <c r="D119" s="19"/>
-      <c r="E119" s="19"/>
-      <c r="F119" s="19"/>
-      <c r="G119" s="19"/>
-      <c r="H119" s="19"/>
-      <c r="I119" s="19"/>
-      <c r="J119" s="19"/>
-      <c r="K119" s="19"/>
-      <c r="L119" s="19"/>
-      <c r="M119" s="19"/>
-      <c r="N119" s="19"/>
-      <c r="O119" s="19"/>
-      <c r="P119" s="19"/>
-      <c r="Q119" s="19"/>
-      <c r="R119" s="19"/>
-      <c r="S119" s="19"/>
-      <c r="T119" s="19"/>
-      <c r="U119" s="19"/>
-      <c r="V119" s="19"/>
-      <c r="W119" s="19"/>
-      <c r="X119" s="19"/>
-      <c r="Y119" s="19"/>
+      <c r="C119" s="108" t="s">
+        <v>239</v>
+      </c>
+      <c r="D119" s="15"/>
+      <c r="E119" s="15"/>
+      <c r="F119" s="15"/>
+      <c r="G119" s="15"/>
+      <c r="H119" s="15"/>
+      <c r="I119" s="15"/>
+      <c r="J119" s="15"/>
+      <c r="K119" s="15"/>
+      <c r="L119" s="15"/>
+      <c r="M119" s="15"/>
+      <c r="N119" s="15"/>
+      <c r="O119" s="15"/>
+      <c r="P119" s="15"/>
+      <c r="Q119" s="15"/>
+      <c r="R119" s="15"/>
+      <c r="S119" s="15"/>
+      <c r="T119" s="15"/>
+      <c r="U119" s="15"/>
+      <c r="V119" s="15"/>
     </row>
     <row r="120" ht="27.75" customHeight="1">
-      <c r="A120" s="94" t="s">
-        <v>239</v>
+      <c r="A120" s="93" t="s">
+        <v>240</v>
       </c>
       <c r="B120" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="C120" s="109" t="s">
         <v>241</v>
+      </c>
+      <c r="C120" s="108" t="s">
+        <v>140</v>
       </c>
       <c r="D120" s="15"/>
       <c r="E120" s="15"/>
@@ -7317,19 +6951,16 @@
       <c r="T120" s="15"/>
       <c r="U120" s="15"/>
       <c r="V120" s="15"/>
-      <c r="W120" s="15"/>
-      <c r="X120" s="15"/>
-      <c r="Y120" s="15"/>
     </row>
     <row r="121" ht="27.75" customHeight="1">
-      <c r="A121" s="94" t="s">
+      <c r="A121" s="34" t="s">
         <v>242</v>
       </c>
       <c r="B121" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="C121" s="109" t="s">
-        <v>140</v>
+      <c r="C121" s="108" t="s">
+        <v>244</v>
       </c>
       <c r="D121" s="15"/>
       <c r="E121" s="15"/>
@@ -7350,51 +6981,43 @@
       <c r="T121" s="15"/>
       <c r="U121" s="15"/>
       <c r="V121" s="15"/>
-      <c r="W121" s="15"/>
-      <c r="X121" s="15"/>
-      <c r="Y121" s="15"/>
     </row>
     <row r="122" ht="27.75" customHeight="1">
       <c r="A122" s="34" t="s">
-        <v>244</v>
-      </c>
-      <c r="B122" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="C122" s="109" t="s">
+      <c r="B122" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C122" s="14"/>
+      <c r="D122" s="19"/>
+      <c r="E122" s="19"/>
+      <c r="F122" s="19"/>
+      <c r="G122" s="19"/>
+      <c r="H122" s="19"/>
+      <c r="I122" s="19"/>
+      <c r="J122" s="19"/>
+      <c r="K122" s="19"/>
+      <c r="L122" s="19"/>
+      <c r="M122" s="19"/>
+      <c r="N122" s="19"/>
+      <c r="O122" s="19"/>
+      <c r="P122" s="19"/>
+      <c r="Q122" s="19"/>
+      <c r="R122" s="19"/>
+      <c r="S122" s="19"/>
+      <c r="T122" s="19"/>
+      <c r="U122" s="19"/>
+      <c r="V122" s="19"/>
+    </row>
+    <row r="123" ht="27.75" customHeight="1">
+      <c r="A123" s="38" t="s">
         <v>246</v>
       </c>
-      <c r="D122" s="15"/>
-      <c r="E122" s="15"/>
-      <c r="F122" s="15"/>
-      <c r="G122" s="15"/>
-      <c r="H122" s="15"/>
-      <c r="I122" s="15"/>
-      <c r="J122" s="15"/>
-      <c r="K122" s="15"/>
-      <c r="L122" s="15"/>
-      <c r="M122" s="15"/>
-      <c r="N122" s="15"/>
-      <c r="O122" s="15"/>
-      <c r="P122" s="15"/>
-      <c r="Q122" s="15"/>
-      <c r="R122" s="15"/>
-      <c r="S122" s="15"/>
-      <c r="T122" s="15"/>
-      <c r="U122" s="15"/>
-      <c r="V122" s="15"/>
-      <c r="W122" s="15"/>
-      <c r="X122" s="15"/>
-      <c r="Y122" s="15"/>
-    </row>
-    <row r="123" ht="27.75" customHeight="1">
-      <c r="A123" s="34" t="s">
-        <v>247</v>
-      </c>
-      <c r="B123" s="35" t="s">
-        <v>21</v>
-      </c>
-      <c r="C123" s="14"/>
+      <c r="B123" s="96" t="s">
+        <v>195</v>
+      </c>
+      <c r="C123" s="33"/>
       <c r="D123" s="19"/>
       <c r="E123" s="19"/>
       <c r="F123" s="19"/>
@@ -7414,78 +7037,69 @@
       <c r="T123" s="19"/>
       <c r="U123" s="19"/>
       <c r="V123" s="19"/>
-      <c r="W123" s="19"/>
-      <c r="X123" s="19"/>
-      <c r="Y123" s="19"/>
-    </row>
-    <row r="124" ht="27.75" customHeight="1">
-      <c r="A124" s="38" t="s">
+    </row>
+    <row r="124" ht="33" customHeight="1">
+      <c r="A124" s="97" t="s">
+        <v>196</v>
+      </c>
+      <c r="B124" s="69" t="s">
+        <v>247</v>
+      </c>
+      <c r="C124" s="33"/>
+      <c r="D124" s="84"/>
+      <c r="E124" s="84"/>
+      <c r="F124" s="84"/>
+      <c r="G124" s="84"/>
+      <c r="H124" s="84"/>
+      <c r="I124" s="84"/>
+      <c r="J124" s="84"/>
+      <c r="K124" s="84"/>
+      <c r="L124" s="84"/>
+      <c r="M124" s="84"/>
+      <c r="N124" s="84"/>
+      <c r="O124" s="84"/>
+      <c r="P124" s="84"/>
+      <c r="Q124" s="84"/>
+      <c r="R124" s="84"/>
+      <c r="S124" s="84"/>
+      <c r="T124" s="84"/>
+      <c r="U124" s="84"/>
+      <c r="V124" s="84"/>
+    </row>
+    <row r="125" ht="27.75" customHeight="1">
+      <c r="A125" s="34">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="B125" s="44" t="s">
         <v>248</v>
       </c>
-      <c r="B124" s="97" t="s">
-        <v>195</v>
-      </c>
-      <c r="C124" s="33"/>
-      <c r="D124" s="19"/>
-      <c r="E124" s="19"/>
-      <c r="F124" s="19"/>
-      <c r="G124" s="19"/>
-      <c r="H124" s="19"/>
-      <c r="I124" s="19"/>
-      <c r="J124" s="19"/>
-      <c r="K124" s="19"/>
-      <c r="L124" s="19"/>
-      <c r="M124" s="19"/>
-      <c r="N124" s="19"/>
-      <c r="O124" s="19"/>
-      <c r="P124" s="19"/>
-      <c r="Q124" s="19"/>
-      <c r="R124" s="19"/>
-      <c r="S124" s="19"/>
-      <c r="T124" s="19"/>
-      <c r="U124" s="19"/>
-      <c r="V124" s="19"/>
-      <c r="W124" s="19"/>
-      <c r="X124" s="19"/>
-      <c r="Y124" s="19"/>
-    </row>
-    <row r="125" ht="33" customHeight="1">
-      <c r="A125" s="98" t="s">
-        <v>196</v>
-      </c>
-      <c r="B125" s="69" t="s">
-        <v>249</v>
-      </c>
       <c r="C125" s="33"/>
-      <c r="D125" s="84"/>
-      <c r="E125" s="84"/>
-      <c r="F125" s="84"/>
-      <c r="G125" s="84"/>
-      <c r="H125" s="84"/>
-      <c r="I125" s="84"/>
-      <c r="J125" s="84"/>
-      <c r="K125" s="84"/>
-      <c r="L125" s="84"/>
-      <c r="M125" s="84"/>
-      <c r="N125" s="84"/>
-      <c r="O125" s="84"/>
-      <c r="P125" s="84"/>
-      <c r="Q125" s="84"/>
-      <c r="R125" s="84"/>
-      <c r="S125" s="84"/>
-      <c r="T125" s="84"/>
-      <c r="U125" s="84"/>
-      <c r="V125" s="84"/>
-      <c r="W125" s="84"/>
-      <c r="X125" s="84"/>
-      <c r="Y125" s="84"/>
-    </row>
-    <row r="126" ht="27.75" customHeight="1">
-      <c r="A126" s="34">
-        <v>0.67708333333333337</v>
-      </c>
-      <c r="B126" s="44" t="s">
-        <v>250</v>
+      <c r="D125" s="19"/>
+      <c r="E125" s="19"/>
+      <c r="F125" s="19"/>
+      <c r="G125" s="19"/>
+      <c r="H125" s="19"/>
+      <c r="I125" s="19"/>
+      <c r="J125" s="19"/>
+      <c r="K125" s="19"/>
+      <c r="L125" s="19"/>
+      <c r="M125" s="19"/>
+      <c r="N125" s="19"/>
+      <c r="O125" s="19"/>
+      <c r="P125" s="19"/>
+      <c r="Q125" s="19"/>
+      <c r="R125" s="19"/>
+      <c r="S125" s="19"/>
+      <c r="T125" s="19"/>
+      <c r="U125" s="19"/>
+      <c r="V125" s="19"/>
+    </row>
+    <row r="126" ht="29.25" customHeight="1">
+      <c r="A126" s="99">
+        <v>0.6875</v>
+      </c>
+      <c r="B126" s="100" t="s">
+        <v>200</v>
       </c>
       <c r="C126" s="33"/>
       <c r="D126" s="19"/>
@@ -7507,43 +7121,9 @@
       <c r="T126" s="19"/>
       <c r="U126" s="19"/>
       <c r="V126" s="19"/>
-      <c r="W126" s="19"/>
-      <c r="X126" s="19"/>
-      <c r="Y126" s="19"/>
-    </row>
-    <row r="127" ht="29.25" customHeight="1">
-      <c r="A127" s="100">
-        <v>0.6875</v>
-      </c>
-      <c r="B127" s="101" t="s">
-        <v>200</v>
-      </c>
-      <c r="C127" s="33"/>
-      <c r="D127" s="19"/>
-      <c r="E127" s="19"/>
-      <c r="F127" s="19"/>
-      <c r="G127" s="19"/>
-      <c r="H127" s="19"/>
-      <c r="I127" s="19"/>
-      <c r="J127" s="19"/>
-      <c r="K127" s="19"/>
-      <c r="L127" s="19"/>
-      <c r="M127" s="19"/>
-      <c r="N127" s="19"/>
-      <c r="O127" s="19"/>
-      <c r="P127" s="19"/>
-      <c r="Q127" s="19"/>
-      <c r="R127" s="19"/>
-      <c r="S127" s="19"/>
-      <c r="T127" s="19"/>
-      <c r="U127" s="19"/>
-      <c r="V127" s="19"/>
-      <c r="W127" s="19"/>
-      <c r="X127" s="19"/>
-      <c r="Y127" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="50">
+  <mergeCells count="49">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="B6:C6"/>
@@ -7573,7 +7153,6 @@
     <mergeCell ref="A71:C71"/>
     <mergeCell ref="B73:C73"/>
     <mergeCell ref="B74:C74"/>
-    <mergeCell ref="D75:F76"/>
     <mergeCell ref="B85:C85"/>
     <mergeCell ref="B88:C88"/>
     <mergeCell ref="A89:A92"/>
@@ -7589,11 +7168,11 @@
     <mergeCell ref="B107:C107"/>
     <mergeCell ref="B111:C111"/>
     <mergeCell ref="B117:C117"/>
-    <mergeCell ref="B119:C119"/>
+    <mergeCell ref="B118:C118"/>
+    <mergeCell ref="B123:C123"/>
     <mergeCell ref="B124:C124"/>
     <mergeCell ref="B125:C125"/>
     <mergeCell ref="B126:C126"/>
-    <mergeCell ref="B127:C127"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>